<commit_message>
Status report 10 Oct: CI is green again (PR #132 run, 12:09 UTC)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MvTNEvR2SbP4iWxB91Q5Qh
</commit_message>
<xml_diff>
--- a/docs/gokesari-audit/GOKESARI_FEATURE_STATUS_REPORT_2026-10-10.xlsx
+++ b/docs/gokesari-audit/GOKESARI_FEATURE_STATUS_REPORT_2026-10-10.xlsx
@@ -2077,10 +2077,10 @@
         </is>
       </c>
     </row>
-    <row r="86" ht="54" customHeight="1" s="24">
+    <row r="86" ht="42" customHeight="1" s="24">
       <c r="A86" s="39" t="inlineStr">
         <is>
-          <t>6. GitHub Actions stopped starting jobs at 18:04 UTC 9 Oct (billing): #124 to #131 were released without CI on the owner's instruction, and no sandbox payment or nightly test-database backup ran. Jobs started again at 11:48 UTC 10 Oct: the re-run on main @a6862c2 (release #129) passed typecheck, lint and the mobile job, with the unit and integration tests still running at the time of this report; the current head 0ec63f3 (#131) has no CI run yet (Blockers #37).</t>
+          <t>6. GitHub Actions stopped starting jobs at 18:04 UTC 9 Oct (billing): #124 to #131 were released without CI on the owner's instruction, and no sandbox payment or nightly test-database backup ran. Jobs started again at 11:48 UTC 10 Oct: CI is green again - PR #132 (the production code at 0ec63f3 plus this report) passed typecheck, lint, unit and integration tests, the production build and the mobile job at 12:09 UTC (Blockers #37).</t>
         </is>
       </c>
     </row>
@@ -21517,7 +21517,7 @@
       </c>
       <c r="Q215" s="34" t="inlineStr">
         <is>
-          <t>GitHub Actions stopped starting jobs at 18:04 UTC on 9 Oct (billing / spending limit): #124 to #131 merged without CI on the owner's instruction (local tsc, eslint, next build and Vitest 1,662 passed for #124). Jobs started again at 11:48 UTC on 10 Oct (re-runs on staging and main): the re-run on main @a6862c2 (release #129) passed typecheck, lint and the mobile job, with the unit and integration tests still running at the time of this report; the current head 0ec63f3 (#131) has no CI run yet (Blockers #37).</t>
+          <t>GitHub Actions stopped starting jobs at 18:04 UTC on 9 Oct (billing / spending limit): #124 to #131 merged without CI on the owner's instruction (local tsc, eslint, next build and Vitest 1,662 passed for #124). Jobs started again at 11:48 UTC on 10 Oct (re-runs on staging and main): CI is green again - PR #132 (the production code at 0ec63f3 plus this report) passed typecheck, lint, unit and integration tests, the production build and the mobile job at 12:09 UTC (Blockers #37).</t>
         </is>
       </c>
       <c r="R215" s="34" t="inlineStr">
@@ -41126,7 +41126,7 @@
         </is>
       </c>
     </row>
-    <row r="31" ht="87" customHeight="1" s="24">
+    <row r="31" ht="75" customHeight="1" s="24">
       <c r="A31" s="32" t="n">
         <v>30</v>
       </c>
@@ -41142,7 +41142,7 @@
       </c>
       <c r="D31" s="34" t="inlineStr">
         <is>
-          <t>CI on the staging merge of #104 (docs only) failed in 'Unit and integration tests'; the same code passed on the PR head and on 6f3c28f. Investigate the failing test / re-run before the next staging merge. 10 Oct: superseded by #37 - no CI ran from 9 Oct 18:04 UTC; re-runs on staging and main started 11:48 UTC 10 Oct (the re-run on main @a6862c2 (release #129) passed typecheck, lint and the mobile job, with the unit and integration tests still running at the time of this report; the current head 0ec63f3 (#131) has no CI run yet).</t>
+          <t>CI on the staging merge of #104 (docs only) failed in 'Unit and integration tests'; the same code passed on the PR head and on 6f3c28f. Investigate the failing test / re-run before the next staging merge. 10 Oct: resolved - CI is green again - PR #132 (the production code at 0ec63f3 plus this report) passed typecheck, lint, unit and integration tests, the production build and the mobile job at 12:09 UTC.</t>
         </is>
       </c>
       <c r="E31" s="34" t="inlineStr">
@@ -41157,7 +41157,7 @@
       </c>
       <c r="G31" s="34" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Resolved</t>
         </is>
       </c>
       <c r="H31" s="34" t="inlineStr">
@@ -41422,7 +41422,7 @@
       </c>
       <c r="D38" s="34" t="inlineStr">
         <is>
-          <t>From 9 Oct 18:04 UTC no CI, no Sandbox payment runs and no nightly Test database backup (run 22 failed). #124 to #131 were merged without CI on the owner's instruction. Jobs started again 11:48 UTC 10 Oct: the re-run on main @a6862c2 (release #129) passed typecheck, lint and the mobile job, with the unit and integration tests still running at the time of this report; the current head 0ec63f3 (#131) has no CI run yet. Next: CI green on main, re-run the Test database backup, then the two sandbox payments (C-01, S-13).</t>
+          <t>From 9 Oct 18:04 UTC no CI, no Sandbox payment runs and no nightly Test database backup (run 22 failed). #124 to #131 were merged without CI on the owner's instruction. Jobs started again 11:48 UTC 10 Oct: CI is green again - PR #132 (the production code at 0ec63f3 plus this report) passed typecheck, lint, unit and integration tests, the production build and the mobile job at 12:09 UTC. Next: re-run the Test database backup, then the two sandbox payments (C-01, S-13).</t>
         </is>
       </c>
       <c r="E38" s="34" t="inlineStr">

</xml_diff>